<commit_message>
sprint details update and Us3 update (milestone3)
</commit_message>
<xml_diff>
--- a/SE202526/Management/Sprint7/BurndownSprint7.xlsx
+++ b/SE202526/Management/Sprint7/BurndownSprint7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\IdeaProjects\MindustryGroupProjectPrivate\SE202526\Management\Sprint7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47644BC2-2E44-499E-BB8B-7F3A8468449E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8872E8C-97B4-4CE3-ADAC-3530621CB960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Sprint Burndown Chart</t>
   </si>
@@ -86,9 +86,6 @@
     <t>Acabar de implementar o gerador de mapa semanal</t>
   </si>
   <si>
-    <t>0.5</t>
-  </si>
-  <si>
     <t>Acabar de implementar a parte do Terramoto e Tsunami</t>
   </si>
   <si>
@@ -117,9 +114,6 @@
   </si>
   <si>
     <t>Day 11</t>
-  </si>
-  <si>
-    <t>1.5</t>
   </si>
 </sst>
 </file>
@@ -1007,10 +1001,10 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1156,10 +1150,10 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1719,14 +1713,14 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="50" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3" s="48"/>
       <c r="G3" s="48"/>
       <c r="H3" s="48"/>
       <c r="I3" s="51"/>
       <c r="J3" s="50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K3" s="48"/>
       <c r="L3" s="48"/>
@@ -1805,16 +1799,16 @@
         <v>11</v>
       </c>
       <c r="L5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="M5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="N5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="N5" s="9" t="s">
-        <v>23</v>
-      </c>
       <c r="O5" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="2:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1852,7 +1846,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" s="19">
         <v>5</v>
@@ -1884,7 +1878,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D8" s="19">
         <v>3</v>
@@ -1910,7 +1904,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" s="40">
         <v>6</v>
@@ -1942,7 +1936,7 @@
         <v>5</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="19">
         <v>3</v>
@@ -1954,16 +1948,16 @@
       <c r="I10" s="22"/>
       <c r="J10" s="23"/>
       <c r="K10" s="21"/>
-      <c r="L10" s="21" t="s">
-        <v>16</v>
-      </c>
+      <c r="L10" s="21"/>
       <c r="M10" s="21">
         <v>1</v>
       </c>
-      <c r="N10" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="21"/>
+      <c r="N10" s="21">
+        <v>1</v>
+      </c>
+      <c r="O10" s="21">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="2:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="17">
@@ -2173,11 +2167,11 @@
       </c>
       <c r="N20" s="29">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="29">
         <f t="shared" ref="O20" si="2">SUM(O6:O19)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="2:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2227,11 +2221,11 @@
       </c>
       <c r="N21" s="36">
         <f t="shared" ref="N21:O21" si="6">M21-SUM(N6:N19)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="36">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>